<commit_message>
Add Teams contact list generator and review report
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 10:45</t>
+          <t>Generated 29 Mar 2026 11:04</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 10:45</t>
+          <t>Generated 29 Mar 2026 11:04</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 10:45</t>
+          <t>Generated 29 Mar 2026 11:04</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 10:45</t>
+          <t>Generated 29 Mar 2026 11:04</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 10:45</t>
+          <t>Generated 29 Mar 2026 11:04</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 10:45</t>
+          <t>Generated 29 Mar 2026 11:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve Teams match labels and footnotes
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:04</t>
+          <t>Generated 29 Mar 2026 11:10</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,11 @@
           <t>Sam Rush</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -704,7 +708,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
@@ -718,23 +722,371 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>*** Fuzzy = matched by the cautious fuzzy fallback after exact and override-based matching failed.</t>
+          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | B Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generated 29 Mar 2026 11:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Georgina Riches</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>07710475970</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>fam.riches@btinternet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Cath Pearson</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>07803 177572</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>cath.pearson@ntlworld.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Charlene Jacobs</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>No Match</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Diane Doyle</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>07944 757679</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>dianeldoyle@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Jacquie Conway</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>07900333359</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>jacquie.conway@outlook.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Joan Mc Crossan</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>07739708728</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>jemccrossan@aol.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Liz Long</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>07711 603036</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>lizzylong1@btinternet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Sally Charlton</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>07724 103325</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>sallycharlton22@btinternet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Sue white</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>01256 893013</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>susan582009@hotmail.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -754,14 +1106,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | B Squad</t>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | C Squad</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:04</t>
+          <t>Generated 29 Mar 2026 11:10</t>
         </is>
       </c>
     </row>
@@ -805,7 +1157,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Georgina Riches</t>
+          <t>Kate Liggett</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
@@ -816,12 +1168,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>07710475970</t>
+          <t>07913406561</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>fam.riches@btinternet.com</t>
+          <t>kate.liggett80@gmail.com</t>
         </is>
       </c>
     </row>
@@ -829,7 +1181,7 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Cath Pearson</t>
+          <t>Alison Jameson</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
@@ -840,12 +1192,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07803 177572</t>
+          <t>07593 569268</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>cath.pearson@ntlworld.com</t>
+          <t>alison.jameson@gmail.com</t>
         </is>
       </c>
     </row>
@@ -853,23 +1205,31 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Charlene Jacobs</t>
+          <t>Joanne Stanley</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>No Match</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>07754 115078</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>joanneecairns@hotmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Diane Doyle</t>
+          <t>Katherine Rogers</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr"/>
@@ -880,12 +1240,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07944 757679</t>
+          <t>07885 304570</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>dianeldoyle@gmail.com</t>
+          <t>katherinerogers10@gmail.com</t>
         </is>
       </c>
     </row>
@@ -893,7 +1253,7 @@
       <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Jacquie Conway</t>
+          <t>Kim Field</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr"/>
@@ -904,12 +1264,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07900333359</t>
+          <t>07500 660820</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>jacquie.conway@outlook.com</t>
+          <t>kimfield65@gmail.com</t>
         </is>
       </c>
     </row>
@@ -917,7 +1277,7 @@
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Joan Mc Crossan</t>
+          <t>Lynn McKenzie</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr"/>
@@ -928,12 +1288,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>07739708728</t>
+          <t>07887 522574</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>jemccrossan@aol.com</t>
+          <t>Lynnmckenzie@live.co.uk</t>
         </is>
       </c>
     </row>
@@ -941,10 +1301,14 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Liz Long</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
+          <t>Trish Harris</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Not Signed Up</t>
@@ -952,661 +1316,65 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>07711 603036</t>
+          <t>07801966381</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>lizzylong1@btinternet.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Sally Charlton</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>07724 103325</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>sallycharlton22@btinternet.com</t>
+          <t>harrisstrish@outlook.com</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Sue white</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>01256 893013</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>susan582009@hotmail.co.uk</t>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>*** Fuzzy = matched by the cautious fuzzy fallback after exact and override-based matching failed.</t>
+          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | C Squad</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Generated 29 Mar 2026 11:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Captain</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Kate Liggett</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>07913406561</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>kate.liggett80@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Alison Jameson</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>07593 569268</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>alison.jameson@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Joanne Stanley</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>07754 115078</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>joanneecairns@hotmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Katherine Rogers</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>07885 304570</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>katherinerogers10@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Kim Field</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>07500 660820</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>kimfield65@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Lynn McKenzie</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>07887 522574</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Lynnmckenzie@live.co.uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Trish Harris</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>07801966381</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>harrisstrish@outlook.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>* Not Signed Up = exact name matched in club records, but no current paid 2026 membership was found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>*** Fuzzy = matched by the cautious fuzzy fallback after exact and override-based matching failed.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A12:F12"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | D Squad</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Generated 29 Mar 2026 11:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Captain</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Susie Cooke</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>07742396206</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>susie.cooke@icloud.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Alicia Freimuth</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>07941038211</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>alicia.freimuth@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Carol- Anne Harrison</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>07799624958</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>cah.dbf@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Clare Bambridge</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>07973838412</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>clare.bambridge@outlook.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Fran Jones</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>07765 140012</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>fran.999.jones@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Juliet Worthington</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>07810358292</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>juliet_worthington@hotmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Sarah Gibbons</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>07837 418366</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>nandsgibbons@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Susan Gilchrist</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>07802 574286</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>mrs.susan.gilchrist@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>* Not Signed Up = exact name matched in club records, but no current paid 2026 membership was found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>*** Fuzzy = matched by the cautious fuzzy fallback after exact and override-based matching failed.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A15:F15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1626,14 +1394,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | E Squad</t>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | D Squad</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:04</t>
+          <t>Generated 29 Mar 2026 11:10</t>
         </is>
       </c>
     </row>
@@ -1677,23 +1445,23 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Sue White</t>
+          <t>Susie Cooke</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>01256 893013</t>
+          <t>07742396206</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>susan582009@hotmail.co.uk</t>
+          <t>susie.cooke@icloud.com</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1469,7 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Claire Taylor</t>
+          <t>Alicia Freimuth</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
@@ -1712,12 +1480,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07792410799</t>
+          <t>07941038211</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>clairechicago1@gmail.com</t>
+          <t>alicia.freimuth@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1725,27 +1493,23 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Helen Eyres</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
+          <t>Carol- Anne Harrison</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>07801107701</t>
+          <t>07799624958</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>helen_eyers@yahoo.co.uk</t>
+          <t>cah.dbf@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1753,23 +1517,23 @@
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Jax S B</t>
+          <t>Clare Bambridge</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07889433872</t>
+          <t>07973838412</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>jaxsb1962@gmail.com</t>
+          <t>clare.bambridge@outlook.com</t>
         </is>
       </c>
     </row>
@@ -1777,23 +1541,23 @@
       <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Jessica Palmer</t>
+          <t>Fran Jones</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07962260856</t>
+          <t>07765 140012</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>JESSICA.PALMER@FLITEPARTNERS.COM</t>
+          <t>fran.999.jones@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1565,7 @@
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Jo Baines</t>
+          <t>Juliet Worthington</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr"/>
@@ -1812,12 +1576,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>07789 882500</t>
+          <t>07810358292</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>bainesfamily@ntlworld.com</t>
+          <t>juliet_worthington@hotmail.com</t>
         </is>
       </c>
     </row>
@@ -1825,27 +1589,23 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Lindsey Evans</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
+          <t>Sarah Gibbons</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>07973 826745</t>
+          <t>07837 418366</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>lindsay@myevans.com</t>
+          <t>nandsgibbons@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1853,6 +1613,330 @@
       <c r="A11" s="5" t="inlineStr"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
+          <t>Susan Gilchrist</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>07802 574286</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>mrs.susan.gilchrist@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | E Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generated 29 Mar 2026 11:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Sue White</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>01256 893013</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>susan582009@hotmail.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Claire Taylor</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>07792410799</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>clairechicago1@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Helen Eyres</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>07801107701</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>helen_eyers@yahoo.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Jax S B</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>07889433872</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>jaxsb1962@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Jessica Palmer</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>07962260856</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>JESSICA.PALMER@FLITEPARTNERS.COM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Jo Baines</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>07789 882500</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>bainesfamily@ntlworld.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Lindsey Evans</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>07973 826745</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>lindsay@myevans.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
           <t>Liz Gruenstern</t>
         </is>
       </c>
@@ -1924,7 +2008,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
@@ -1938,16 +2022,32 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>*** Fuzzy = matched by the cautious fuzzy fallback after exact and override-based matching failed.</t>
+          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1960,7 +2060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1981,7 +2081,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:04</t>
+          <t>Generated 29 Mar 2026 11:10</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2124,11 @@
           <t>Becky Cockerill</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Not Signed Up</t>
@@ -2092,7 +2196,11 @@
           <t>Mo Clackett</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -2140,7 +2248,11 @@
           <t>Val Rowlands</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -2184,7 +2296,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
@@ -2198,17 +2310,33 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>*** Fuzzy = matched by the cautious fuzzy fallback after exact and override-based matching failed.</t>
+          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Best Fit match markers to Teams outputs
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:10</t>
+          <t>Generated 29 Mar 2026 11:15</t>
         </is>
       </c>
     </row>
@@ -722,31 +722,39 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
@@ -755,6 +763,646 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | B Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generated 29 Mar 2026 11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Georgina Riches</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>07710475970</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>fam.riches@btinternet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Cath Pearson</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>07803 177572</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>cath.pearson@ntlworld.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Charlene Jacobs</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>No Match</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Diane Doyle</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>07944 757679</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>dianeldoyle@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Jacquie Conway</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>07900333359</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>jacquie.conway@outlook.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Joan Mc Crossan</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Best Fit</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>07739708728</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>jemccrossan@aol.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Liz Long</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>07711 603036</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>lizzylong1@btinternet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Sally Charlton</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>07724 103325</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>sallycharlton22@btinternet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Sue white</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>01256 893013</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>susan582009@hotmail.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | C Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generated 29 Mar 2026 11:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Kate Liggett</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>07913406561</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>kate.liggett80@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Alison Jameson</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>07593 569268</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>alison.jameson@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Joanne Stanley</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>07754 115078</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>joanneecairns@hotmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Katherine Rogers</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>07885 304570</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>katherinerogers10@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Kim Field</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>07500 660820</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>kimfield65@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Lynn McKenzie</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>07887 522574</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Lynnmckenzie@live.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Trish Harris</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>07801966381</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>harrisstrish@outlook.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -774,14 +1422,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | B Squad</t>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | D Squad</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:10</t>
+          <t>Generated 29 Mar 2026 11:15</t>
         </is>
       </c>
     </row>
@@ -825,7 +1473,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Georgina Riches</t>
+          <t>Susie Cooke</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
@@ -836,12 +1484,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>07710475970</t>
+          <t>07742396206</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>fam.riches@btinternet.com</t>
+          <t>susie.cooke@icloud.com</t>
         </is>
       </c>
     </row>
@@ -849,23 +1497,23 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Cath Pearson</t>
+          <t>Alicia Freimuth</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07803 177572</t>
+          <t>07941038211</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>cath.pearson@ntlworld.com</t>
+          <t>alicia.freimuth@gmail.com</t>
         </is>
       </c>
     </row>
@@ -873,23 +1521,31 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Charlene Jacobs</t>
+          <t>Carol- Anne Harrison</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>No Match</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>07799624958</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>cah.dbf@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Diane Doyle</t>
+          <t>Clare Bambridge</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr"/>
@@ -900,12 +1556,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07944 757679</t>
+          <t>07973838412</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>dianeldoyle@gmail.com</t>
+          <t>clare.bambridge@outlook.com</t>
         </is>
       </c>
     </row>
@@ -913,14 +1569,10 @@
       <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Jacquie Conway</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
+          <t>Fran Jones</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -928,12 +1580,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07900333359</t>
+          <t>07765 140012</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>jacquie.conway@outlook.com</t>
+          <t>fran.999.jones@gmail.com</t>
         </is>
       </c>
     </row>
@@ -941,23 +1593,23 @@
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Joan Mc Crossan</t>
+          <t>Juliet Worthington</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>07739708728</t>
+          <t>07810358292</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>jemccrossan@aol.com</t>
+          <t>juliet_worthington@hotmail.com</t>
         </is>
       </c>
     </row>
@@ -965,23 +1617,23 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Liz Long</t>
+          <t>Sarah Gibbons</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>07711 603036</t>
+          <t>07837 418366</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>lizzylong1@btinternet.com</t>
+          <t>nandsgibbons@gmail.com</t>
         </is>
       </c>
     </row>
@@ -989,7 +1641,7 @@
       <c r="A11" s="5" t="inlineStr"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Sally Charlton</t>
+          <t>Susan Gilchrist</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr"/>
@@ -1000,82 +1652,62 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>07724 103325</t>
+          <t>07802 574286</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>sallycharlton22@btinternet.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Sue white</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>01256 893013</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>susan582009@hotmail.co.uk</t>
+          <t>mrs.susan.gilchrist@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A17:F17"/>
@@ -1086,13 +1718,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1106,14 +1738,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | C Squad</t>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | E Squad</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:10</t>
+          <t>Generated 29 Mar 2026 11:15</t>
         </is>
       </c>
     </row>
@@ -1157,23 +1789,27 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Kate Liggett</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
+          <t>Sue White</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>07913406561</t>
+          <t>01256 893013</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>kate.liggett80@gmail.com</t>
+          <t>susan582009@hotmail.co.uk</t>
         </is>
       </c>
     </row>
@@ -1181,23 +1817,23 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Alison Jameson</t>
+          <t>Claire Taylor</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07593 569268</t>
+          <t>07792410799</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>alison.jameson@gmail.com</t>
+          <t>clairechicago1@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1205,23 +1841,27 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Joanne Stanley</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
+          <t>Helen Eyres</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>07754 115078</t>
+          <t>07801107701</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>joanneecairns@hotmail.com</t>
+          <t>helen_eyers@yahoo.co.uk</t>
         </is>
       </c>
     </row>
@@ -1229,23 +1869,27 @@
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Katherine Rogers</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
+          <t>Jax S B</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07885 304570</t>
+          <t>07889433872</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>katherinerogers10@gmail.com</t>
+          <t>jaxsb1962@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1253,23 +1897,23 @@
       <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Kim Field</t>
+          <t>Jessica Palmer</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07500 660820</t>
+          <t>07962260856</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>kimfield65@gmail.com</t>
+          <t>JESSICA.PALMER@FLITEPARTNERS.COM</t>
         </is>
       </c>
     </row>
@@ -1277,23 +1921,23 @@
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Lynn McKenzie</t>
+          <t>Jo Baines</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>07887 522574</t>
+          <t>07789 882500</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Lynnmckenzie@live.co.uk</t>
+          <t>bainesfamily@ntlworld.com</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1945,7 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Trish Harris</t>
+          <t>Lindsey Evans</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1316,65 +1960,145 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>07801966381</t>
+          <t>07973 826745</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>harrisstrish@outlook.com</t>
+          <t>lindsay@myevans.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Liz Gruenstern</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>07769867559</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>liz.gruenstern@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Maew Tatam</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>07885719965</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>walanda@hotmail.com</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+      <c r="A13" s="5" t="inlineStr"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Vicky Judge</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>07775 683165</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>vixtiger1@icloud.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A20:F20"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1394,14 +2118,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | D Squad</t>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | Reserves</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:10</t>
+          <t>Generated 29 Mar 2026 11:15</t>
         </is>
       </c>
     </row>
@@ -1438,30 +2162,30 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Susie Cooke</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Becky Cockerill</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Not Signed Up</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>07742396206</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>susie.cooke@icloud.com</t>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>07876 352111</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>beckyandstuart@btinternet.com</t>
         </is>
       </c>
     </row>
@@ -1469,47 +2193,43 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Alicia Freimuth</t>
+          <t>Jane Woods</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>07941038211</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>alicia.freimuth@gmail.com</t>
-        </is>
-      </c>
+          <t>No Match</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Carol- Anne Harrison</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
+          <t>Jill Penton</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>07799624958</t>
+          <t>07845 144977</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>cah.dbf@gmail.com</t>
+          <t>jillian.penton@virginmedia.com</t>
         </is>
       </c>
     </row>
@@ -1517,10 +2237,14 @@
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Clare Bambridge</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
+          <t>Mo Clackett</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -1528,12 +2252,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07973838412</t>
+          <t>07703 196204</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>clare.bambridge@outlook.com</t>
+          <t>moclackett@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1541,7 +2265,7 @@
       <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Fran Jones</t>
+          <t>Pauline Snell</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr"/>
@@ -1552,12 +2276,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07765 140012</t>
+          <t>07877300234</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>fran.999.jones@gmail.com</t>
+          <t>psnell66@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1565,10 +2289,14 @@
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Juliet Worthington</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
+          <t>Val Rowlands</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -1576,12 +2304,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>07810358292</t>
+          <t>07891572164</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>juliet_worthington@hotmail.com</t>
+          <t>valrowlands@aol.co.uk</t>
         </is>
       </c>
     </row>
@@ -1589,7 +2317,7 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Sarah Gibbons</t>
+          <t>Val Talbot</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr"/>
@@ -1600,741 +2328,65 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>07837 418366</t>
+          <t>07767 072546</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>nandsgibbons@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Susan Gilchrist</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>07802 574286</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>mrs.susan.gilchrist@gmail.com</t>
+          <t>valerie.talbot@ntlworld.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A15:F15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | E Squad</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Generated 29 Mar 2026 11:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Captain</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Sue White</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>01256 893013</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>susan582009@hotmail.co.uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Claire Taylor</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>07792410799</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>clairechicago1@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Helen Eyres</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>07801107701</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>helen_eyers@yahoo.co.uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Jax S B</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Override</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>07889433872</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>jaxsb1962@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Jessica Palmer</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>07962260856</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>JESSICA.PALMER@FLITEPARTNERS.COM</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Jo Baines</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>07789 882500</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>bainesfamily@ntlworld.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Lindsey Evans</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>07973 826745</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>lindsay@myevans.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Liz Gruenstern</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>07769867559</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>liz.gruenstern@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Maew Tatam</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>07885719965</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>walanda@hotmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Vicky Judge</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>07775 683165</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>vixtiger1@icloud.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | Reserves</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Generated 29 Mar 2026 11:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Captain</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr"/>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Becky Cockerill</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>07876 352111</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>beckyandstuart@btinternet.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Jane Woods</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>No Match</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Jill Penton</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>07845 144977</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>jillian.penton@virginmedia.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Mo Clackett</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>07703 196204</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>moclackett@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Pauline Snell</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>07877300234</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>psnell66@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Val Rowlands</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>07891572164</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>valrowlands@aol.co.uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Val Talbot</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>07767 072546</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>valerie.talbot@ntlworld.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>*** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>**** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>***** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>

</xml_diff>

<commit_message>
Generate one team PDF per output file
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:15</t>
+          <t>Generated 29 Mar 2026 12:50</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:15</t>
+          <t>Generated 29 Mar 2026 12:50</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:15</t>
+          <t>Generated 29 Mar 2026 12:50</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:15</t>
+          <t>Generated 29 Mar 2026 12:50</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:15</t>
+          <t>Generated 29 Mar 2026 12:50</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 11:15</t>
+          <t>Generated 29 Mar 2026 12:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Import ClubSpark Main Contacts and use for Teams juniors
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 12:50</t>
+          <t>Generated 30 Mar 2026 14:35</t>
         </is>
       </c>
     </row>
@@ -548,14 +548,26 @@
           <t>Jane Dow</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>No Match</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr"/>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>+447721967512</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>janeatimmis@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr"/>
@@ -572,12 +584,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07962 260856</t>
+          <t>07962260856</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>jessica.palmer@flitepartners.com</t>
+          <t>JESSICA.PALMER@FLITEPARTNERS.COM</t>
         </is>
       </c>
     </row>
@@ -789,7 +801,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 12:50</t>
+          <t>Generated 30 Mar 2026 14:35</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1145,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 12:50</t>
+          <t>Generated 30 Mar 2026 14:35</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1441,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 12:50</t>
+          <t>Generated 30 Mar 2026 14:35</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1757,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 12:50</t>
+          <t>Generated 30 Mar 2026 14:35</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2137,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 29 Mar 2026 12:50</t>
+          <t>Generated 30 Mar 2026 14:35</t>
         </is>
       </c>
     </row>
@@ -2196,14 +2208,26 @@
           <t>Jane Woods</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>No Match</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>07578 331340</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>ajanewoods@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update Teams outputs and workflow actions
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 30 Mar 2026 14:35</t>
+          <t>Generated 31 Mar 2026 15:53</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 30 Mar 2026 14:35</t>
+          <t>Generated 31 Mar 2026 15:53</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 30 Mar 2026 14:35</t>
+          <t>Generated 31 Mar 2026 15:53</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 30 Mar 2026 14:35</t>
+          <t>Generated 31 Mar 2026 15:53</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 30 Mar 2026 14:35</t>
+          <t>Generated 31 Mar 2026 15:53</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 30 Mar 2026 14:35</t>
+          <t>Generated 31 Mar 2026 15:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add member email preview flow and refresh Teams outputs
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -109,10 +109,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -501,7 +501,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 31 Mar 2026 15:53</t>
+          <t>Generated 01 Apr 2026 09:52</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07962260856</t>
+          <t>07962 260856</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>JESSICA.PALMER@FLITEPARTNERS.COM</t>
+          <t>jessica.palmer@flitepartners.com</t>
         </is>
       </c>
     </row>
@@ -632,12 +632,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07973 684940</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>leilawarwick@me.com</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -660,12 +660,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07765 164044</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>samrush336@gmail.com</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -759,8 +759,15 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:F13"/>
@@ -768,6 +775,7 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -775,6 +783,662 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | B Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generated 01 Apr 2026 09:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Georgina Riches</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>07710475970</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>fam.riches@btinternet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Cath Pearson</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>07803 177572</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>cath.pearson@ntlworld.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Charlene Jacobs</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>No Match</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Diane Doyle</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>07944 757679</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>dianeldoyle@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Jacquie Conway</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>07900333359</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>jacquie.conway@outlook.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Joan Mc Crossan</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Best Fit</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>07739708728</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>jemccrossan@aol.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Liz Long</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Sally Charlton</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>07724 103325</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>sallycharlton22@btinternet.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Sue white</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | C Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generated 01 Apr 2026 09:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Kate Liggett</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>07913406561</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>kate.liggett80@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Alison Jameson</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>07593 569268</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>alison.jameson@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Joanne Stanley</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>07754 115078</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>joanneecairns@hotmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Katherine Rogers</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Kim Field</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>07500 660820</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>kimfield65@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Lynn McKenzie</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>07887 522574</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Lynnmckenzie@live.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Trish Harris</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>07801966381</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>harrisstrish@outlook.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -794,14 +1458,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | B Squad</t>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | D Squad</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 31 Mar 2026 15:53</t>
+          <t>Generated 01 Apr 2026 09:52</t>
         </is>
       </c>
     </row>
@@ -845,7 +1509,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Georgina Riches</t>
+          <t>Susie Cooke</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
@@ -856,12 +1520,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>07710475970</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>fam.riches@btinternet.com</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -869,23 +1533,23 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Cath Pearson</t>
+          <t>Alicia Freimuth</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07803 177572</t>
+          <t>07941038211</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>cath.pearson@ntlworld.com</t>
+          <t>alicia.freimuth@gmail.com</t>
         </is>
       </c>
     </row>
@@ -893,23 +1557,31 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Charlene Jacobs</t>
+          <t>Carol- Anne Harrison</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>No Match</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>07799624958</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>cah.dbf@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Diane Doyle</t>
+          <t>Clare Bambridge</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr"/>
@@ -920,12 +1592,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07944 757679</t>
+          <t>07973838412</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>dianeldoyle@gmail.com</t>
+          <t>clare.bambridge@outlook.com</t>
         </is>
       </c>
     </row>
@@ -933,14 +1605,10 @@
       <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Jacquie Conway</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
+          <t>Fran Jones</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -948,12 +1616,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07900333359</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>jacquie.conway@outlook.com</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -961,27 +1629,23 @@
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Joan Mc Crossan</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Best Fit</t>
-        </is>
-      </c>
+          <t>Juliet Worthington</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>07739708728</t>
+          <t>07810358292</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>jemccrossan@aol.com</t>
+          <t>juliet_worthington@hotmail.com</t>
         </is>
       </c>
     </row>
@@ -989,23 +1653,23 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Liz Long</t>
+          <t>Sarah Gibbons</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>07711 603036</t>
+          <t>07837 418366</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>lizzylong1@btinternet.com</t>
+          <t>nandsgibbons@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1677,7 @@
       <c r="A11" s="5" t="inlineStr"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Sally Charlton</t>
+          <t>Susan Gilchrist</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr"/>
@@ -1024,91 +1688,71 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>07724 103325</t>
+          <t>07802 574286</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>sallycharlton22@btinternet.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Sue white</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>01256 893013</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>susan582009@hotmail.co.uk</t>
+          <t>mrs.susan.gilchrist@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A18:F18"/>
@@ -1118,13 +1762,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1138,14 +1782,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | C Squad</t>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | E Squad</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 31 Mar 2026 15:53</t>
+          <t>Generated 01 Apr 2026 09:52</t>
         </is>
       </c>
     </row>
@@ -1189,23 +1833,27 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Kate Liggett</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
+          <t>Sue White</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>07913406561</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>kate.liggett80@gmail.com</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -1213,23 +1861,23 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Alison Jameson</t>
+          <t>Claire Taylor</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07593 569268</t>
+          <t>07792410799</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>alison.jameson@gmail.com</t>
+          <t>clairechicago1@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1237,23 +1885,27 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Joanne Stanley</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
+          <t>Helen Eyres</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>07754 115078</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>joanneecairns@hotmail.com</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -1261,23 +1913,27 @@
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Katherine Rogers</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
+          <t>Jax S B</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07885 304570</t>
+          <t>07889433872</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>katherinerogers10@gmail.com</t>
+          <t>jaxsb1962@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1285,23 +1941,23 @@
       <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Kim Field</t>
+          <t>Jessica Palmer</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Not Signed Up</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07500 660820</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>kimfield65@gmail.com</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -1309,23 +1965,23 @@
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Lynn McKenzie</t>
+          <t>Jo Baines</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>07887 522574</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Lynnmckenzie@live.co.uk</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1989,7 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Trish Harris</t>
+          <t>Lindsey Evans</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1343,78 +1999,158 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Liz Gruenstern</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>No Consent</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Maew Tatam</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
           <t>Not Signed Up</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>07801966381</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>harrisstrish@outlook.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>07885719965</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>walanda@hotmail.com</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+      <c r="A13" s="5" t="inlineStr"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Vicky Judge</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>07775 683165</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>vixtiger1@icloud.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
           <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1434,14 +2170,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | D Squad</t>
+          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | Reserves</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 31 Mar 2026 15:53</t>
+          <t>Generated 01 Apr 2026 09:52</t>
         </is>
       </c>
     </row>
@@ -1478,30 +2214,30 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Susie Cooke</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>07742396206</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>susie.cooke@icloud.com</t>
+      <c r="A4" s="5" t="inlineStr"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Becky Cockerill</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>07876 352111</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>beckyandstuart@btinternet.com</t>
         </is>
       </c>
     </row>
@@ -1509,23 +2245,27 @@
       <c r="A5" s="5" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Alicia Freimuth</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
+          <t>Jane Woods</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07941038211</t>
+          <t>07578 331340</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>alicia.freimuth@gmail.com</t>
+          <t>ajanewoods@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1533,23 +2273,27 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Carol- Anne Harrison</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
+          <t>Jill Penton</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fuzzy</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>07799624958</t>
+          <t>07845 144977</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>cah.dbf@gmail.com</t>
+          <t>jillian.penton@virginmedia.com</t>
         </is>
       </c>
     </row>
@@ -1557,10 +2301,14 @@
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Clare Bambridge</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
+          <t>Mo Clackett</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -1568,12 +2316,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>07973838412</t>
+          <t>No Consent</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>clare.bambridge@outlook.com</t>
+          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -1581,7 +2329,7 @@
       <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Fran Jones</t>
+          <t>Pauline Snell</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr"/>
@@ -1592,12 +2340,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>07765 140012</t>
+          <t>07877300234</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>fran.999.jones@gmail.com</t>
+          <t>psnell66@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1605,10 +2353,14 @@
       <c r="A9" s="5" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Juliet Worthington</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
+          <t>Val Rowlands</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Senior</t>
@@ -1616,12 +2368,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>07810358292</t>
+          <t>07891572164</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>juliet_worthington@hotmail.com</t>
+          <t>valrowlands@aol.co.uk</t>
         </is>
       </c>
     </row>
@@ -1629,7 +2381,7 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Sarah Gibbons</t>
+          <t>Val Talbot</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr"/>
@@ -1640,771 +2392,66 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>07837 418366</t>
+          <t>07767 072546</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>nandsgibbons@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Susan Gilchrist</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>07802 574286</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>mrs.susan.gilchrist@gmail.com</t>
+          <t>valerie.talbot@ntlworld.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | E Squad</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Generated 31 Mar 2026 15:53</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Captain</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Sue White</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>01256 893013</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>susan582009@hotmail.co.uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Claire Taylor</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>07792410799</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>clairechicago1@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Helen Eyres</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>07801107701</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>helen_eyers@yahoo.co.uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Jax S B</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Override</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>07889433872</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>jaxsb1962@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Jessica Palmer</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>07962260856</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>JESSICA.PALMER@FLITEPARTNERS.COM</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Jo Baines</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>07789 882500</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>bainesfamily@ntlworld.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Lindsey Evans</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>07973 826745</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>lindsay@myevans.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Liz Gruenstern</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>07769867559</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>liz.gruenstern@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Maew Tatam</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>07885719965</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>walanda@hotmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Vicky Judge</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>07775 683165</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>vixtiger1@icloud.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A15:F15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Avondale Tennis Club | LADIES TEAMS 2026 Summer | Reserves</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Generated 31 Mar 2026 15:53</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Captain</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr"/>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Becky Cockerill</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>07876 352111</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>beckyandstuart@btinternet.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Jane Woods</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Override</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>07578 331340</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>ajanewoods@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Jill Penton</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>07845 144977</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>jillian.penton@virginmedia.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Mo Clackett</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>07703 196204</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>moclackett@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Pauline Snell</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>07877300234</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>psnell66@gmail.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Val Rowlands</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>07891572164</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>valrowlands@aol.co.uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Val Talbot</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>07767 072546</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>valerie.talbot@ntlworld.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:F13"/>
@@ -2412,6 +2459,7 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update team mailout and dashboard tooling
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -44,7 +44,7 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="006B7280"/>
+      <color rgb="001F1F1F"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -480,15 +480,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -501,7 +502,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 01 Apr 2026 09:52</t>
+          <t>Generated 02 Apr 2026 11:51</t>
         </is>
       </c>
     </row>
@@ -518,22 +519,27 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
         </is>
       </c>
     </row>
@@ -550,22 +556,27 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>+447721967512</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>janeatimmis@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
           <t>Override</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>+447721967512</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>janeatimmis@gmail.com</t>
         </is>
       </c>
     </row>
@@ -576,22 +587,30 @@
           <t>Amy Palmer</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Self: Yes
+Parent: No</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>07962 260856</t>
+          <t>Self: 07962 260856
+Parent: 07962260856</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>jessica.palmer@flitepartners.com</t>
-        </is>
-      </c>
+          <t>Self: jessica.palmer@flitepartners.com
+Parent: JESSICA.PALMER@FLITEPARTNERS.COM</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr"/>
@@ -600,10 +619,14 @@
           <t>Jane Vincent</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -616,6 +639,7 @@
           <t>thevincents365@gmail.com</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr"/>
@@ -624,22 +648,27 @@
           <t>Leila Warwick</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
+          <t>07973 684940</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
-        </is>
-      </c>
+          <t>leilawarwick@me.com</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr"/>
@@ -650,22 +679,27 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>07765 164044</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>samrush336@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
           <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -676,10 +710,14 @@
           <t>Sian Thomas</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -692,6 +730,7 @@
           <t>siannie.thomas@icloud.com</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr"/>
@@ -700,10 +739,14 @@
           <t>Wendy Day</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -716,67 +759,68 @@
           <t>W_mudd@yahoo.com</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Consent: No means the captain may use the phone/email for team management, but may not pass it on to anyone else.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>** Not Signed Up = no current membership was found.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+          <t>*** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>**** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>***** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>****** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+          <t>******* Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -788,15 +832,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -809,7 +854,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 01 Apr 2026 09:52</t>
+          <t>Generated 02 Apr 2026 11:51</t>
         </is>
       </c>
     </row>
@@ -826,22 +871,27 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
         </is>
       </c>
     </row>
@@ -856,10 +906,14 @@
           <t>Georgina Riches</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -872,6 +926,7 @@
           <t>fam.riches@btinternet.com</t>
         </is>
       </c>
+      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr"/>
@@ -880,10 +935,14 @@
           <t>Cath Pearson</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -896,6 +955,7 @@
           <t>cath.pearson@ntlworld.com</t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr"/>
@@ -904,14 +964,27 @@
           <t>Charlene Jacobs</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>No Match</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>+447872314523</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>jacobscharlene@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr"/>
@@ -920,10 +993,14 @@
           <t>Diane Doyle</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -936,6 +1013,7 @@
           <t>dianeldoyle@gmail.com</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr"/>
@@ -946,22 +1024,27 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>07900333359</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>jacquie.conway@outlook.com</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
           <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>07900333359</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>jacquie.conway@outlook.com</t>
         </is>
       </c>
     </row>
@@ -974,22 +1057,27 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>07739708728</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>jemccrossan@aol.com</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
           <t>Best Fit</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>07739708728</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>jemccrossan@aol.com</t>
         </is>
       </c>
     </row>
@@ -1000,22 +1088,27 @@
           <t>Liz Long</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
+          <t>07711 603036</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
-        </is>
-      </c>
+          <t>lizzylong1@btinternet.com</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr"/>
@@ -1024,10 +1117,14 @@
           <t>Sally Charlton</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1040,6 +1137,7 @@
           <t>sallycharlton22@btinternet.com</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr"/>
@@ -1050,85 +1148,90 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>01256 893013</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>susan582009@hotmail.co.uk</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
           <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Consent: No means the captain may use the phone/email for team management, but may not pass it on to anyone else.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>** Not Signed Up = no current membership was found.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+          <t>*** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>**** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>***** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>****** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+          <t>******* Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A19:G19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1140,15 +1243,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1161,7 +1265,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 01 Apr 2026 09:52</t>
+          <t>Generated 02 Apr 2026 11:51</t>
         </is>
       </c>
     </row>
@@ -1178,22 +1282,27 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
         </is>
       </c>
     </row>
@@ -1208,10 +1317,14 @@
           <t>Kate Liggett</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1224,6 +1337,7 @@
           <t>kate.liggett80@gmail.com</t>
         </is>
       </c>
+      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr"/>
@@ -1232,10 +1346,14 @@
           <t>Alison Jameson</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1248,6 +1366,7 @@
           <t>alison.jameson@gmail.com</t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr"/>
@@ -1256,10 +1375,14 @@
           <t>Joanne Stanley</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1272,6 +1395,7 @@
           <t>joanneecairns@hotmail.com</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr"/>
@@ -1280,22 +1404,27 @@
           <t>Katherine Rogers</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
+          <t>07885 304570</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
-        </is>
-      </c>
+          <t>katherinerogers10@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr"/>
@@ -1304,10 +1433,14 @@
           <t>Kim Field</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1320,6 +1453,7 @@
           <t>kimfield65@gmail.com</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr"/>
@@ -1328,10 +1462,14 @@
           <t>Lynn McKenzie</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1344,6 +1482,7 @@
           <t>Lynnmckenzie@live.co.uk</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr"/>
@@ -1354,85 +1493,90 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>07801966381</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>harrisstrish@outlook.com</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
           <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>07801966381</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>harrisstrish@outlook.com</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Consent: No means the captain may use the phone/email for team management, but may not pass it on to anyone else.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>** Not Signed Up = no current membership was found.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+          <t>*** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>**** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>***** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>****** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+          <t>******* Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1444,15 +1588,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1465,7 +1610,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 01 Apr 2026 09:52</t>
+          <t>Generated 02 Apr 2026 11:51</t>
         </is>
       </c>
     </row>
@@ -1482,22 +1627,27 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
         </is>
       </c>
     </row>
@@ -1512,22 +1662,27 @@
           <t>Susie Cooke</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>No Consent</t>
+          <t>07742396206</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>No Consent</t>
-        </is>
-      </c>
+          <t>susie.cooke@icloud.com</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr"/>
@@ -1536,10 +1691,14 @@
           <t>Alicia Freimuth</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1552,6 +1711,7 @@
           <t>alicia.freimuth@gmail.com</t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr"/>
@@ -1560,10 +1720,14 @@
           <t>Carol- Anne Harrison</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1576,6 +1740,7 @@
           <t>cah.dbf@gmail.com</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr"/>
@@ -1584,10 +1749,14 @@
           <t>Clare Bambridge</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1600,6 +1769,7 @@
           <t>clare.bambridge@outlook.com</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr"/>
@@ -1608,22 +1778,27 @@
           <t>Fran Jones</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
+          <t>07765 140012</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
-        </is>
-      </c>
+          <t>fran.999.jones@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr"/>
@@ -1632,10 +1807,14 @@
           <t>Juliet Worthington</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1648,6 +1827,7 @@
           <t>juliet_worthington@hotmail.com</t>
         </is>
       </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr"/>
@@ -1656,10 +1836,14 @@
           <t>Sarah Gibbons</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1672,6 +1856,7 @@
           <t>nandsgibbons@gmail.com</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr"/>
@@ -1680,10 +1865,14 @@
           <t>Susan Gilchrist</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1696,67 +1885,68 @@
           <t>mrs.susan.gilchrist@gmail.com</t>
         </is>
       </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Consent: No means the captain may use the phone/email for team management, but may not pass it on to anyone else.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>** Not Signed Up = no current membership was found.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+          <t>*** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>**** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>***** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>****** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+          <t>******* Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A19:G19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1768,15 +1958,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1789,7 +1980,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 01 Apr 2026 09:52</t>
+          <t>Generated 02 Apr 2026 11:51</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1997,27 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
         </is>
       </c>
     </row>
@@ -1838,22 +2034,27 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>01256 893013</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>susan582009@hotmail.co.uk</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
           <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>No Consent</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -1864,10 +2065,14 @@
           <t>Claire Taylor</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1880,6 +2085,7 @@
           <t>clairechicago1@gmail.com</t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr"/>
@@ -1890,22 +2096,27 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>07801107701</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>helen_eyers@yahoo.co.uk</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
           <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -1918,22 +2129,27 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>07889433872</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>jaxsb1962@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
           <t>Override</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Not Signed Up</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>07889433872</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>jaxsb1962@gmail.com</t>
         </is>
       </c>
     </row>
@@ -1944,22 +2160,27 @@
           <t>Jessica Palmer</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
+          <t>07962260856</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
-        </is>
-      </c>
+          <t>JESSICA.PALMER@FLITEPARTNERS.COM</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr"/>
@@ -1968,22 +2189,27 @@
           <t>Jo Baines</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
+          <t>07789 882500</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
-        </is>
-      </c>
+          <t>bainesfamily@ntlworld.com</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr"/>
@@ -1994,22 +2220,27 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>07973 826745</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>lindsay@myevans.com</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
           <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -2020,22 +2251,27 @@
           <t>Liz Gruenstern</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
+          <t>07769867559</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>No Consent</t>
-        </is>
-      </c>
+          <t>liz.gruenstern@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr"/>
@@ -2044,10 +2280,14 @@
           <t>Maew Tatam</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -2060,6 +2300,7 @@
           <t>walanda@hotmail.com</t>
         </is>
       </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr"/>
@@ -2068,10 +2309,14 @@
           <t>Vicky Judge</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr"/>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Not Signed Up</t>
+        </is>
+      </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -2084,67 +2329,68 @@
           <t>vixtiger1@icloud.com</t>
         </is>
       </c>
+      <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Consent: No means the captain may use the phone/email for team management, but may not pass it on to anyone else.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>** Not Signed Up = no current membership was found.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+          <t>*** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>**** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>***** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>****** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+          <t>******* Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A19:G19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2156,15 +2402,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2177,7 +2424,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 01 Apr 2026 09:52</t>
+          <t>Generated 02 Apr 2026 11:51</t>
         </is>
       </c>
     </row>
@@ -2194,22 +2441,27 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>Match</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Email</t>
         </is>
       </c>
     </row>
@@ -2222,22 +2474,27 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>07876 352111</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>beckyandstuart@btinternet.com</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
           <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>07876 352111</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>beckyandstuart@btinternet.com</t>
         </is>
       </c>
     </row>
@@ -2250,22 +2507,27 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>07578 331340</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>ajanewoods@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
           <t>Override</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>07578 331340</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>ajanewoods@gmail.com</t>
         </is>
       </c>
     </row>
@@ -2278,22 +2540,27 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>07845 144977</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>jillian.penton@virginmedia.com</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
           <t>Fuzzy</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>07845 144977</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>jillian.penton@virginmedia.com</t>
         </is>
       </c>
     </row>
@@ -2306,22 +2573,27 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>07703 196204</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>moclackett@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
           <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>No Consent</t>
         </is>
       </c>
     </row>
@@ -2332,10 +2604,14 @@
           <t>Pauline Snell</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -2348,6 +2624,7 @@
           <t>psnell66@gmail.com</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr"/>
@@ -2358,22 +2635,27 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
+          <t>Senior</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>07891572164</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>valrowlands@aol.co.uk</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
           <t>Nickname</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Senior</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>07891572164</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>valrowlands@aol.co.uk</t>
         </is>
       </c>
     </row>
@@ -2384,10 +2666,14 @@
           <t>Val Talbot</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Senior</t>
+        </is>
+      </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -2400,67 +2686,68 @@
           <t>valerie.talbot@ntlworld.com</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>* Not Signed Up = exact or resolved name matched in club records, but no current paid 2026 membership was found.</t>
+          <t>* Consent: No means the captain may use the phone/email for team management, but may not pass it on to anyone else.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>** No Match = no unique exact-name match was found in current club member/contact records.</t>
+          <t>** Not Signed Up = no current membership was found.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>*** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
+          <t>*** No Match = no unique exact-name match was found in current club member/contact records.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>**** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
+          <t>**** Best Fit = one row was chosen from several exact-name candidates using the best available contact evidence.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>***** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
+          <t>***** Override = resolved by an explicit override; this usually represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>****** Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
+          <t>****** Nickname = resolved by a short-name or nickname rule; this may also represent a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>******* No Consent = the current contact record does not allow contact details to be shared, so phone and email are withheld.</t>
+          <t>******* Fuzzy = resolved by the cautious fuzzy fallback; this represents a typo or misspelling in the source data.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: fix regx for Hi payer
</commit_message>
<xml_diff>
--- a/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
+++ b/Teams/generated/LADIES TEAMS 2026 Summer - Contact Lists.xlsx
@@ -502,7 +502,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 02 Apr 2026 11:51</t>
+          <t>Generated 02 Apr 2026 14:17</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 02 Apr 2026 11:51</t>
+          <t>Generated 02 Apr 2026 14:17</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 02 Apr 2026 11:51</t>
+          <t>Generated 02 Apr 2026 14:17</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Not Signed Up</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1610,7 +1610,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 02 Apr 2026 11:51</t>
+          <t>Generated 02 Apr 2026 14:17</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 02 Apr 2026 11:51</t>
+          <t>Generated 02 Apr 2026 14:17</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 02 Apr 2026 11:51</t>
+          <t>Generated 02 Apr 2026 14:17</t>
         </is>
       </c>
     </row>

</xml_diff>